<commit_message>
Debit Advice uploading AR Type
</commit_message>
<xml_diff>
--- a/uploads/UPLOAD-TEMPLATE/DEBIT-ADVICE-SALES-COLLECTION-INVENTORY-UPLOAD-TEMPLATE.xlsx
+++ b/uploads/UPLOAD-TEMPLATE/DEBIT-ADVICE-SALES-COLLECTION-INVENTORY-UPLOAD-TEMPLATE.xlsx
@@ -5,16 +5,21 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kacruz\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6784312-C30B-4C64-99AC-9A6A7C4AF30F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F334F5D-3B59-4AA2-90D9-B99234712714}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00008A2C-D6BB-4F78-94C4-BCFBAE050A86}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="TRANSACTION" sheetId="1" r:id="rId1"/>
+    <sheet name="ADVANCES_AR TYPE" sheetId="2" r:id="rId2"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">TRANSACTION!$A$1:$H$1</definedName>
+    <definedName name="AdvancesARTypeList">'ADVANCES_AR TYPE'!$A$2:$A$1000</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -34,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="40">
   <si>
     <t>GL</t>
   </si>
@@ -58,6 +63,102 @@
   </si>
   <si>
     <t>AMOUNT</t>
+  </si>
+  <si>
+    <t>ADVANCES - AGENCY</t>
+  </si>
+  <si>
+    <t>ADVANCES - BROKER</t>
+  </si>
+  <si>
+    <t>ADVANCES - CICIP</t>
+  </si>
+  <si>
+    <t>ADVANCES - CHICK IN CHECK IN PAYMENT</t>
+  </si>
+  <si>
+    <t>ADVANCES - CONTRACT BREEDER</t>
+  </si>
+  <si>
+    <t>ADVANCES - DOC FREIGHT</t>
+  </si>
+  <si>
+    <t>ADVANCES - FEED INGREDIENTS</t>
+  </si>
+  <si>
+    <t>ADVANCES - FEEDMILL TOLLING</t>
+  </si>
+  <si>
+    <t>ADVANCES - GROWER</t>
+  </si>
+  <si>
+    <t>ADVANCES - GROWER A1</t>
+  </si>
+  <si>
+    <t>ADVANCES - LAND ACQUISITION</t>
+  </si>
+  <si>
+    <t>ADVANCES - LESSOR</t>
+  </si>
+  <si>
+    <t>ADVANCES - SUBCONTRACTOR</t>
+  </si>
+  <si>
+    <t>ADVANCES - SUPPLIERS</t>
+  </si>
+  <si>
+    <t>ADVANCES - TELEGRAPHIC</t>
+  </si>
+  <si>
+    <t>ADVANCES - TRUCKER</t>
+  </si>
+  <si>
+    <t>ADVANCES - VACMED</t>
+  </si>
+  <si>
+    <t>ADVANCES TO EMPLOYEES</t>
+  </si>
+  <si>
+    <t>AR EMPLOYEES (BANK LOANS)</t>
+  </si>
+  <si>
+    <t>AR EMPLOYEES (CAR LOAN)</t>
+  </si>
+  <si>
+    <t>AR EMPLOYEES (DM CHARGES)</t>
+  </si>
+  <si>
+    <t>AR EMPLOYEES (GYM)</t>
+  </si>
+  <si>
+    <t>AR EMPLOYEES (HMO DEPENDENTS)</t>
+  </si>
+  <si>
+    <t>AR EMPLOYEES (RFID CHARGES)</t>
+  </si>
+  <si>
+    <t>AR EMPLOYEES (SALARY LOAN)</t>
+  </si>
+  <si>
+    <t>AR EMPLOYEES (TELEPHONE)</t>
+  </si>
+  <si>
+    <t>CLAIMS - MATERNITY</t>
+  </si>
+  <si>
+    <t>CLAIMS - SICKNESS</t>
+  </si>
+  <si>
+    <t>CLAIMS - VEHICLE INSURANCE</t>
+  </si>
+  <si>
+    <t>CODE</t>
+  </si>
+  <si>
+    <t>NAME</t>
+  </si>
+  <si>
+    <t>ADVANCES/AR TYPE</t>
   </si>
 </sst>
 </file>
@@ -67,7 +168,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.000"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -89,8 +190,13 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Carlito"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -103,8 +209,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF2CC"/>
+        <bgColor rgb="FF000000"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -112,11 +224,26 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -136,6 +263,15 @@
     <xf numFmtId="164" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -450,21 +586,22 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{58DACE88-7F71-4361-A307-FFBC7051559A}">
-  <dimension ref="A1:H1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:I19"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="10.42578125" style="2" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="3.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="5.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.42578125" style="1" customWidth="1"/>
+    <col min="4" max="4" width="11.42578125" style="1" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="19" style="1" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="14.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="9.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="52" style="1" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="9.42578125" style="3" bestFit="1" customWidth="1"/>
-    <col min="9" max="16384" width="9.140625" style="2"/>
+    <col min="9" max="9" width="33" style="2" bestFit="1" customWidth="1"/>
+    <col min="10" max="16384" width="9.140625" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9">
       <c r="A1" s="4" t="s">
         <v>1</v>
       </c>
@@ -489,10 +626,407 @@
       <c r="H1" s="6" t="s">
         <v>7</v>
       </c>
-    </row>
+      <c r="I1" s="11" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9">
+      <c r="A2" s="7"/>
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
+      <c r="G2" s="2"/>
+      <c r="H2" s="2"/>
+    </row>
+    <row r="3" spans="1:9">
+      <c r="A3" s="7"/>
+      <c r="B3" s="2"/>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2"/>
+      <c r="F3" s="2"/>
+      <c r="G3" s="2"/>
+      <c r="H3" s="2"/>
+    </row>
+    <row r="4" spans="1:9">
+      <c r="A4" s="8"/>
+      <c r="B4" s="2"/>
+      <c r="C4" s="2"/>
+      <c r="D4" s="2"/>
+      <c r="E4" s="2"/>
+      <c r="F4" s="2"/>
+      <c r="G4" s="2"/>
+      <c r="H4" s="2"/>
+    </row>
+    <row r="5" spans="1:9">
+      <c r="A5" s="8"/>
+      <c r="B5" s="2"/>
+      <c r="C5" s="2"/>
+      <c r="D5" s="2"/>
+      <c r="E5" s="2"/>
+      <c r="F5" s="2"/>
+      <c r="G5" s="2"/>
+      <c r="H5" s="2"/>
+    </row>
+    <row r="6" spans="1:9">
+      <c r="B6" s="2"/>
+      <c r="C6" s="2"/>
+      <c r="D6" s="2"/>
+      <c r="E6" s="2"/>
+      <c r="F6" s="2"/>
+      <c r="G6" s="2"/>
+      <c r="H6" s="2"/>
+    </row>
+    <row r="7" spans="1:9">
+      <c r="B7" s="2"/>
+      <c r="C7" s="2"/>
+      <c r="D7" s="2"/>
+      <c r="E7" s="2"/>
+      <c r="F7" s="2"/>
+      <c r="G7" s="2"/>
+      <c r="H7" s="2"/>
+    </row>
+    <row r="8" spans="1:9">
+      <c r="B8" s="2"/>
+      <c r="C8" s="2"/>
+      <c r="D8" s="2"/>
+      <c r="E8" s="2"/>
+      <c r="F8" s="2"/>
+      <c r="G8" s="2"/>
+      <c r="H8" s="2"/>
+    </row>
+    <row r="9" spans="1:9">
+      <c r="B9" s="2"/>
+      <c r="C9" s="2"/>
+      <c r="D9" s="2"/>
+      <c r="E9" s="2"/>
+      <c r="F9" s="2"/>
+      <c r="G9" s="2"/>
+      <c r="H9" s="2"/>
+    </row>
+    <row r="10" spans="1:9">
+      <c r="B10" s="2"/>
+      <c r="C10" s="2"/>
+      <c r="D10" s="2"/>
+      <c r="E10" s="2"/>
+      <c r="F10" s="2"/>
+      <c r="G10" s="2"/>
+      <c r="H10" s="2"/>
+    </row>
+    <row r="11" spans="1:9">
+      <c r="B11" s="2"/>
+      <c r="C11" s="2"/>
+      <c r="D11" s="2"/>
+      <c r="E11" s="2"/>
+      <c r="F11" s="2"/>
+      <c r="G11" s="2"/>
+      <c r="H11" s="2"/>
+    </row>
+    <row r="12" spans="1:9">
+      <c r="B12" s="2"/>
+      <c r="C12" s="2"/>
+      <c r="D12" s="2"/>
+      <c r="E12" s="2"/>
+      <c r="F12" s="2"/>
+      <c r="G12" s="2"/>
+      <c r="H12" s="2"/>
+    </row>
+    <row r="13" spans="1:9">
+      <c r="B13" s="2"/>
+      <c r="C13" s="2"/>
+      <c r="D13" s="2"/>
+      <c r="E13" s="2"/>
+      <c r="F13" s="2"/>
+      <c r="G13" s="2"/>
+      <c r="H13" s="2"/>
+    </row>
+    <row r="14" spans="1:9">
+      <c r="B14" s="2"/>
+      <c r="C14" s="2"/>
+      <c r="D14" s="2"/>
+      <c r="E14" s="2"/>
+      <c r="F14" s="2"/>
+      <c r="G14" s="2"/>
+      <c r="H14" s="2"/>
+    </row>
+    <row r="15" spans="1:9">
+      <c r="B15" s="2"/>
+      <c r="C15" s="2"/>
+      <c r="D15" s="2"/>
+      <c r="E15" s="2"/>
+      <c r="F15" s="2"/>
+      <c r="G15" s="2"/>
+      <c r="H15" s="2"/>
+    </row>
+    <row r="16" spans="1:9">
+      <c r="B16" s="2"/>
+      <c r="C16" s="2"/>
+      <c r="D16" s="2"/>
+      <c r="E16" s="2"/>
+      <c r="F16" s="2"/>
+      <c r="G16" s="2"/>
+      <c r="H16" s="2"/>
+    </row>
+    <row r="17" s="2" customFormat="1"/>
+    <row r="18" s="2" customFormat="1"/>
+    <row r="19" s="2" customFormat="1"/>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I2:I1089" xr:uid="{CFA8CD00-804C-4435-91BB-8C6A8D001B65}">
+      <formula1>AdvancesARTypeList</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="200" verticalDpi="200" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2D8AF88D-AFEA-4C18-84CC-264888798359}">
+  <dimension ref="A1:B29"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="33" style="9" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="38.5703125" style="9" bestFit="1" customWidth="1"/>
+    <col min="3" max="16384" width="9.140625" style="9"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2">
+      <c r="A1" s="10" t="s">
+        <v>37</v>
+      </c>
+      <c r="B1" s="10" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" s="10" t="s">
+        <v>8</v>
+      </c>
+      <c r="B2" s="10" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2">
+      <c r="A3" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" s="10" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2">
+      <c r="A4" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4" s="10" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2">
+      <c r="A5" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" s="10" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2">
+      <c r="A6" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="B6" s="10" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2">
+      <c r="A7" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="B7" s="10" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2">
+      <c r="A8" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="B8" s="10" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2">
+      <c r="A9" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="B9" s="10" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2">
+      <c r="A10" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="B10" s="10" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2">
+      <c r="A11" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="B11" s="10" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2">
+      <c r="A12" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="B12" s="10" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2">
+      <c r="A13" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="B13" s="10" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2">
+      <c r="A14" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="B14" s="10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2">
+      <c r="A15" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="B15" s="10" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2">
+      <c r="A16" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="B16" s="10" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2">
+      <c r="A17" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="B17" s="10" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2">
+      <c r="A18" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="B18" s="10" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2">
+      <c r="A19" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="B19" s="10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2">
+      <c r="A20" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="B20" s="10" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2">
+      <c r="A21" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="B21" s="10" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2">
+      <c r="A22" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="B22" s="10" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2">
+      <c r="A23" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="B23" s="10" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2">
+      <c r="A24" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="B24" s="10" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2">
+      <c r="A25" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="B25" s="10" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2">
+      <c r="A26" s="10" t="s">
+        <v>33</v>
+      </c>
+      <c r="B26" s="10" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2">
+      <c r="A27" s="10" t="s">
+        <v>34</v>
+      </c>
+      <c r="B27" s="10" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2">
+      <c r="A28" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="B28" s="10" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2">
+      <c r="A29" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="B29" s="10" t="s">
+        <v>36</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Module Name integration instead of module id
</commit_message>
<xml_diff>
--- a/uploads/UPLOAD-TEMPLATE/DEBIT-ADVICE-SALES-COLLECTION-INVENTORY-UPLOAD-TEMPLATE.xlsx
+++ b/uploads/UPLOAD-TEMPLATE/DEBIT-ADVICE-SALES-COLLECTION-INVENTORY-UPLOAD-TEMPLATE.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F334F5D-3B59-4AA2-90D9-B99234712714}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A146078B-71D9-4A4B-BCF7-1F717B96EDA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00008A2C-D6BB-4F78-94C4-BCFBAE050A86}"/>
   </bookViews>
@@ -168,7 +168,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.000"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -192,11 +192,19 @@
     </font>
     <font>
       <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <color rgb="FF000000"/>
-      <name val="Carlito"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -207,12 +215,6 @@
       <patternFill patternType="solid">
         <fgColor theme="1"/>
         <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFF2CC"/>
-        <bgColor rgb="FF000000"/>
       </patternFill>
     </fill>
   </fills>
@@ -263,15 +265,11 @@
     <xf numFmtId="164" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -586,8 +584,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{58DACE88-7F71-4361-A307-FFBC7051559A}">
-  <dimension ref="A1:I19"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
+  <dimension ref="A1:I2"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.42578125" style="2" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="10.5703125" style="1" bestFit="1" customWidth="1"/>
@@ -595,13 +593,13 @@
     <col min="4" max="4" width="11.42578125" style="1" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="19" style="1" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="14.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="52" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.28515625" style="1" customWidth="1"/>
     <col min="8" max="8" width="9.42578125" style="3" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="33" style="2" bestFit="1" customWidth="1"/>
     <col min="10" max="16384" width="9.140625" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
         <v>1</v>
       </c>
@@ -626,156 +624,19 @@
       <c r="H1" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="11" t="s">
+      <c r="I1" s="8" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="2" spans="1:9">
-      <c r="A2" s="7"/>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
-      <c r="G2" s="2"/>
-      <c r="H2" s="2"/>
-    </row>
-    <row r="3" spans="1:9">
-      <c r="A3" s="7"/>
-      <c r="B3" s="2"/>
-      <c r="C3" s="2"/>
-      <c r="D3" s="2"/>
-      <c r="E3" s="2"/>
-      <c r="F3" s="2"/>
-      <c r="G3" s="2"/>
-      <c r="H3" s="2"/>
-    </row>
-    <row r="4" spans="1:9">
-      <c r="A4" s="8"/>
-      <c r="B4" s="2"/>
-      <c r="C4" s="2"/>
-      <c r="D4" s="2"/>
-      <c r="E4" s="2"/>
-      <c r="F4" s="2"/>
-      <c r="G4" s="2"/>
-      <c r="H4" s="2"/>
-    </row>
-    <row r="5" spans="1:9">
-      <c r="A5" s="8"/>
-      <c r="B5" s="2"/>
-      <c r="C5" s="2"/>
-      <c r="D5" s="2"/>
-      <c r="E5" s="2"/>
-      <c r="F5" s="2"/>
-      <c r="G5" s="2"/>
-      <c r="H5" s="2"/>
-    </row>
-    <row r="6" spans="1:9">
-      <c r="B6" s="2"/>
-      <c r="C6" s="2"/>
-      <c r="D6" s="2"/>
-      <c r="E6" s="2"/>
-      <c r="F6" s="2"/>
-      <c r="G6" s="2"/>
-      <c r="H6" s="2"/>
-    </row>
-    <row r="7" spans="1:9">
-      <c r="B7" s="2"/>
-      <c r="C7" s="2"/>
-      <c r="D7" s="2"/>
-      <c r="E7" s="2"/>
-      <c r="F7" s="2"/>
-      <c r="G7" s="2"/>
-      <c r="H7" s="2"/>
-    </row>
-    <row r="8" spans="1:9">
-      <c r="B8" s="2"/>
-      <c r="C8" s="2"/>
-      <c r="D8" s="2"/>
-      <c r="E8" s="2"/>
-      <c r="F8" s="2"/>
-      <c r="G8" s="2"/>
-      <c r="H8" s="2"/>
-    </row>
-    <row r="9" spans="1:9">
-      <c r="B9" s="2"/>
-      <c r="C9" s="2"/>
-      <c r="D9" s="2"/>
-      <c r="E9" s="2"/>
-      <c r="F9" s="2"/>
-      <c r="G9" s="2"/>
-      <c r="H9" s="2"/>
-    </row>
-    <row r="10" spans="1:9">
-      <c r="B10" s="2"/>
-      <c r="C10" s="2"/>
-      <c r="D10" s="2"/>
-      <c r="E10" s="2"/>
-      <c r="F10" s="2"/>
-      <c r="G10" s="2"/>
-      <c r="H10" s="2"/>
-    </row>
-    <row r="11" spans="1:9">
-      <c r="B11" s="2"/>
-      <c r="C11" s="2"/>
-      <c r="D11" s="2"/>
-      <c r="E11" s="2"/>
-      <c r="F11" s="2"/>
-      <c r="G11" s="2"/>
-      <c r="H11" s="2"/>
-    </row>
-    <row r="12" spans="1:9">
-      <c r="B12" s="2"/>
-      <c r="C12" s="2"/>
-      <c r="D12" s="2"/>
-      <c r="E12" s="2"/>
-      <c r="F12" s="2"/>
-      <c r="G12" s="2"/>
-      <c r="H12" s="2"/>
-    </row>
-    <row r="13" spans="1:9">
-      <c r="B13" s="2"/>
-      <c r="C13" s="2"/>
-      <c r="D13" s="2"/>
-      <c r="E13" s="2"/>
-      <c r="F13" s="2"/>
-      <c r="G13" s="2"/>
-      <c r="H13" s="2"/>
-    </row>
-    <row r="14" spans="1:9">
-      <c r="B14" s="2"/>
-      <c r="C14" s="2"/>
-      <c r="D14" s="2"/>
-      <c r="E14" s="2"/>
-      <c r="F14" s="2"/>
-      <c r="G14" s="2"/>
-      <c r="H14" s="2"/>
-    </row>
-    <row r="15" spans="1:9">
-      <c r="B15" s="2"/>
-      <c r="C15" s="2"/>
-      <c r="D15" s="2"/>
-      <c r="E15" s="2"/>
-      <c r="F15" s="2"/>
-      <c r="G15" s="2"/>
-      <c r="H15" s="2"/>
-    </row>
-    <row r="16" spans="1:9">
-      <c r="B16" s="2"/>
-      <c r="C16" s="2"/>
-      <c r="D16" s="2"/>
-      <c r="E16" s="2"/>
-      <c r="F16" s="2"/>
-      <c r="G16" s="2"/>
-      <c r="H16" s="2"/>
-    </row>
-    <row r="17" s="2" customFormat="1"/>
-    <row r="18" s="2" customFormat="1"/>
-    <row r="19" s="2" customFormat="1"/>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B2" s="9"/>
+      <c r="E2" s="11"/>
+      <c r="F2" s="10"/>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I2:I1089" xr:uid="{CFA8CD00-804C-4435-91BB-8C6A8D001B65}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I2" xr:uid="{CFA8CD00-804C-4435-91BB-8C6A8D001B65}">
       <formula1>AdvancesARTypeList</formula1>
     </dataValidation>
   </dataValidations>
@@ -787,242 +648,241 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2D8AF88D-AFEA-4C18-84CC-264888798359}">
   <dimension ref="A1:B29"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="33" style="9" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="38.5703125" style="9" bestFit="1" customWidth="1"/>
-    <col min="3" max="16384" width="9.140625" style="9"/>
+    <col min="1" max="1" width="33" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="38.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
-      <c r="A1" s="10" t="s">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" s="7" t="s">
         <v>37</v>
       </c>
-      <c r="B1" s="10" t="s">
+      <c r="B1" s="7" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
-      <c r="A2" s="10" t="s">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="B2" s="10" t="s">
+      <c r="B2" s="7" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:2">
-      <c r="A3" s="10" t="s">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="B3" s="10" t="s">
+      <c r="B3" s="7" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:2">
-      <c r="A4" s="10" t="s">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="B4" s="10" t="s">
+      <c r="B4" s="7" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:2">
-      <c r="A5" s="10" t="s">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="B5" s="10" t="s">
+      <c r="B5" s="7" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="1:2">
-      <c r="A6" s="10" t="s">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="B6" s="10" t="s">
+      <c r="B6" s="7" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="7" spans="1:2">
-      <c r="A7" s="10" t="s">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="B7" s="10" t="s">
+      <c r="B7" s="7" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="8" spans="1:2">
-      <c r="A8" s="10" t="s">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="B8" s="10" t="s">
+      <c r="B8" s="7" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="9" spans="1:2">
-      <c r="A9" s="10" t="s">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="B9" s="10" t="s">
+      <c r="B9" s="7" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="10" spans="1:2">
-      <c r="A10" s="10" t="s">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="B10" s="10" t="s">
+      <c r="B10" s="7" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="11" spans="1:2">
-      <c r="A11" s="10" t="s">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="B11" s="10" t="s">
+      <c r="B11" s="7" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="12" spans="1:2">
-      <c r="A12" s="10" t="s">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="B12" s="10" t="s">
+      <c r="B12" s="7" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="13" spans="1:2">
-      <c r="A13" s="10" t="s">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A13" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="B13" s="10" t="s">
+      <c r="B13" s="7" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="14" spans="1:2">
-      <c r="A14" s="10" t="s">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A14" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="B14" s="10" t="s">
+      <c r="B14" s="7" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="15" spans="1:2">
-      <c r="A15" s="10" t="s">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A15" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="B15" s="10" t="s">
+      <c r="B15" s="7" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="16" spans="1:2">
-      <c r="A16" s="10" t="s">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A16" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="B16" s="10" t="s">
+      <c r="B16" s="7" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="17" spans="1:2">
-      <c r="A17" s="10" t="s">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="B17" s="10" t="s">
+      <c r="B17" s="7" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="18" spans="1:2">
-      <c r="A18" s="10" t="s">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A18" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="B18" s="10" t="s">
+      <c r="B18" s="7" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="19" spans="1:2">
-      <c r="A19" s="10" t="s">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A19" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="B19" s="10" t="s">
+      <c r="B19" s="7" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="20" spans="1:2">
-      <c r="A20" s="10" t="s">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A20" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="B20" s="10" t="s">
+      <c r="B20" s="7" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="21" spans="1:2">
-      <c r="A21" s="10" t="s">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A21" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="B21" s="10" t="s">
+      <c r="B21" s="7" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="22" spans="1:2">
-      <c r="A22" s="10" t="s">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A22" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="B22" s="10" t="s">
+      <c r="B22" s="7" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="23" spans="1:2">
-      <c r="A23" s="10" t="s">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A23" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="B23" s="10" t="s">
+      <c r="B23" s="7" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="24" spans="1:2">
-      <c r="A24" s="10" t="s">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A24" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="B24" s="10" t="s">
+      <c r="B24" s="7" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="25" spans="1:2">
-      <c r="A25" s="10" t="s">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A25" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="B25" s="10" t="s">
+      <c r="B25" s="7" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="26" spans="1:2">
-      <c r="A26" s="10" t="s">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A26" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="B26" s="10" t="s">
+      <c r="B26" s="7" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="27" spans="1:2">
-      <c r="A27" s="10" t="s">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A27" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="B27" s="10" t="s">
+      <c r="B27" s="7" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="28" spans="1:2">
-      <c r="A28" s="10" t="s">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A28" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="B28" s="10" t="s">
+      <c r="B28" s="7" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="29" spans="1:2">
-      <c r="A29" s="10" t="s">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A29" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="B29" s="10" t="s">
+      <c r="B29" s="7" t="s">
         <v>36</v>
       </c>
     </row>

</xml_diff>